<commit_message>
docs: record owner decisions on required documents
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/required-documents-draft.xlsx
+++ b/docs/required-documents-draft.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,11 +50,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8D7DA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -89,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -101,9 +96,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -545,15 +537,15 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -579,15 +571,15 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -616,7 +608,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -651,15 +643,15 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -685,15 +677,15 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -719,15 +711,15 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -758,7 +750,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -768,7 +760,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Permit (for example paragraph 11 Tierschutzgesetz) where the local authority requires one; provider confirms in the form, staff check</t>
+          <t>Permit (for example paragraph 11 Tierschutzgesetz) where the local authority requires one. A police certificate is recommended: shown as a hint in the app, no document slot at launch</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -791,7 +783,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -801,12 +793,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Police certificate = extended (paragraph 30a BZRG). First-aid course certificate optional</t>
+          <t>Police certificate = extended (paragraph 30a BZRG)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -834,15 +826,19 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>A police certificate is recommended: shown as a hint in the app, no document slot at launch</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
@@ -866,12 +862,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -900,12 +896,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -934,12 +930,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -968,7 +964,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -980,7 +976,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Craft qualification (Meisterbrief) only if the work is a craft trade that needs one by law (electrics, gas, water, heating); otherwise not needed</t>
+          <t>Proof of certification (craft qualification, for example Meisterbrief) is compulsory, as decided on 28 October</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1003,15 +999,15 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1024,23 +1020,23 @@
       <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>R = required to go live   O = optional (badge when approved)   - = not needed</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>R = required to go live   - = not needed. Optional documents are left out for launch (owner decision, 28 October)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Draft of 28 October 2026 for the owner to approve. Not legal advice: have the German rules checked before launch.</t>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Owner decisions of 28 October 2026 recorded. Not legal advice: have the German rules checked before launch (private persons: tax adviser).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"R,O,-"</formula1>
+      <formula1>"R,-"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1349,7 +1345,11 @@
           <t>Require it from everyone at the start, because Stripe is not built yet</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Yes: photo ID is required from every provider.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1370,7 +1370,11 @@
           <t>Accept the declaration, after the tax adviser agrees</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Private persons submit their ID (in the trade-registration slot) for now. To be confirmed with the tax adviser before launch.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1391,7 +1395,11 @@
           <t>Leave O out for launch (simplest), add the badge later</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Optional documents are left out for launch: every O became not needed.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1412,7 +1420,11 @@
           <t>Optional badge</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>A police certificate is recommended for cleaning and dog walking: shown as a hint, no document slot at launch (not required, no badge).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1433,7 +1445,11 @@
           <t>Add the rule to the service description</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Proof of certification is compulsory for small repairs (craft qualification).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: optional documents get a slot, craft qualification optional for now
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/required-documents-draft.xlsx
+++ b/docs/required-documents-draft.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -96,6 +101,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -537,15 +545,15 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -571,15 +579,15 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -608,7 +616,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -643,15 +651,15 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -677,15 +685,15 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -711,15 +719,15 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -750,7 +758,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>O</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -760,7 +768,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Permit (for example paragraph 11 Tierschutzgesetz) where the local authority requires one. A police certificate is recommended: shown as a hint in the app, no document slot at launch</t>
+          <t>Permit (for example paragraph 11 Tierschutzgesetz) where the local authority requires one. A police certificate is recommended: optional slot, shown as a badge when approved</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -783,7 +791,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -793,12 +801,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>O</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Police certificate = extended (paragraph 30a BZRG)</t>
+          <t>Police certificate = extended (paragraph 30a BZRG). Optional: first-aid course certificate</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -826,17 +834,17 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>A police certificate is recommended: shown as a hint in the app, no document slot at launch</t>
+          <t>A police certificate is recommended: optional slot, shown as a badge when approved</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -862,12 +870,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -896,12 +904,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -930,12 +938,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -964,19 +972,19 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Proof of certification (craft qualification, for example Meisterbrief) is compulsory, as decided on 28 October</t>
+          <t>Craft qualification (for example Meisterbrief) is optional for now, shown as a badge when approved. To be made compulsory later</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -999,15 +1007,15 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1020,23 +1028,23 @@
       <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>R = required to go live   - = not needed. Optional documents are left out for launch (owner decision, 28 October)</t>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>R = required to go live   O = optional (badge when approved)   - = not needed</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Owner decisions of 28 October 2026 recorded. Not legal advice: have the German rules checked before launch (private persons: tax adviser).</t>
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Owner decisions of 28 October 2026 recorded, updated. Not legal advice: have the German rules checked before launch (private persons: tax adviser).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"R,-"</formula1>
+      <formula1>"R,O,-"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1397,7 +1405,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Optional documents are left out for launch: every O became not needed.</t>
+          <t>Optional documents get a slot: shown as a badge when approved, not needed to go live (changed from the first answer on 28 October).</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1430,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>A police certificate is recommended for cleaning and dog walking: shown as a hint, no document slot at launch (not required, no badge).</t>
+          <t>A police certificate is recommended for cleaning and dog walking: an optional slot with a badge.</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1455,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Proof of certification is compulsory for small repairs (craft qualification).</t>
+          <t>Craft qualification is optional for small repairs for now (changed from compulsory); to be made compulsory later.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: trade registration optional for now
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/required-documents-draft.xlsx
+++ b/docs/required-documents-draft.xlsx
@@ -538,9 +538,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -572,9 +572,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -606,9 +606,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -644,9 +644,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -678,9 +678,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -712,9 +712,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -746,9 +746,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -784,9 +784,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -822,9 +822,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -860,9 +860,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -894,9 +894,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -928,9 +928,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -962,9 +962,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1000,9 +1000,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Private persons submit their ID (in the trade-registration slot) for now. To be confirmed with the tax adviser before launch.</t>
+          <t>Trade registration is optional for now (changed on 28 October): private persons (babysitting, dog walking, small household tasks, window cleaning) are not asked for it. Photo ID stays required. Tax adviser to confirm before launch.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Liability insurance optional for now in every category; reminder in README
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/required-documents-draft.xlsx
+++ b/docs/required-documents-draft.xlsx
@@ -611,9 +611,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -751,9 +751,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -827,9 +827,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -865,9 +865,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -899,9 +899,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -933,9 +933,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -967,9 +967,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1297,7 +1297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1436,24 +1436,49 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Liability insurance</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Required for the physical trades (cleaning, gardening, moving, assembly, small repairs, catering, dog walking) in the first table. Can be a hurdle for private persons.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Optional for now, revisit before launch</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Optional for now (28 October). Owner wants a reminder to revisit it later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Craft trades in small repairs</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Electrical, gas, water and heating work needs a Meisterbrief by law. Either add a rule in the service description (no craft trades that need a master qualification) or add a separate category later.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Add the rule to the service description</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Craft qualification is optional for small repairs for now (changed from compulsory); to be made compulsory later.</t>
         </is>

</xml_diff>

<commit_message>
Document requirements per category: required and optional (#18)
* feat: per-category required and optional documents, nine shared document types

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* Trade registration optional for now; photo ID is the only document every category requires

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* Liability insurance optional for now in every category; reminder in README

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* Seeds test: counts for liability insurance optional

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/required-documents-draft.xlsx
+++ b/docs/required-documents-draft.xlsx
@@ -611,9 +611,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -751,9 +751,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -827,9 +827,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -865,9 +865,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -899,9 +899,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -933,9 +933,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -967,9 +967,9 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1297,7 +1297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1436,24 +1436,49 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Liability insurance</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Required for the physical trades (cleaning, gardening, moving, assembly, small repairs, catering, dog walking) in the first table. Can be a hurdle for private persons.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Optional for now, revisit before launch</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Optional for now (28 October). Owner wants a reminder to revisit it later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Craft trades in small repairs</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Electrical, gas, water and heating work needs a Meisterbrief by law. Either add a rule in the service description (no craft trades that need a master qualification) or add a separate category later.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Add the rule to the service description</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Craft qualification is optional for small repairs for now (changed from compulsory); to be made compulsory later.</t>
         </is>

</xml_diff>